<commit_message>
substitude some data from xlsx
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\programing\web\edu\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523DE208-4D93-44E8-91F6-6ECF9D84407B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{404CE13C-8FAF-4444-8021-AE0E7E92B9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{30884FB9-020E-41FA-A013-6B99802F644E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30884FB9-020E-41FA-A013-6B99802F644E}"/>
   </bookViews>
   <sheets>
     <sheet name="website" sheetId="2" r:id="rId1"/>
@@ -39,24 +39,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>主標題</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>副標題</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>icon</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>介紹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>創辦人</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -73,10 +65,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>SubTitle</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>BackgroundPic</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -93,16 +81,34 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Introduction</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>FounderIntroduction</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>websiteTitle</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dataImages\aboutUs\success-story.jpg</t>
+  </si>
+  <si>
+    <t>LongIntro</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ShortIntro</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Title</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>middleLogo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dataImages\middleLogo.png</t>
   </si>
 </sst>
 </file>
@@ -160,14 +166,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -505,22 +508,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D563F2B-87E7-4475-823C-C6BA693017D8}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
         <v>15</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{1025D2D0-FEB9-405F-A577-4B55E6E69442}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -541,28 +558,28 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" t="s">
+      <c r="H1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
         <v>9</v>
-      </c>
-      <c r="F1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -570,20 +587,22 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" t="s">
         <v>3</v>
-      </c>
-      <c r="E2" s="2"/>
-      <c r="H2" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -594,6 +613,9 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{0D8CF109-EFB4-4522-9A9D-9D8AADB9C198}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
a big commit, leave the old multi-page web as lagacy.html and create a single-page one. delete many parts. connect probably all content with data.xlsx.
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,142 +1,248 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\programing\web\edu\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\programing\web\educenter-bootstrap-main\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{404CE13C-8FAF-4444-8021-AE0E7E92B9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C829AC4-F7EF-4CC2-8725-F8987063524C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30884FB9-020E-41FA-A013-6B99802F644E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="website" sheetId="2" r:id="rId1"/>
-    <sheet name="aboutUs" sheetId="1" r:id="rId2"/>
-    <sheet name="previousEvent" sheetId="3" r:id="rId3"/>
-    <sheet name="course" sheetId="4" r:id="rId4"/>
+    <sheet name="website" sheetId="1" r:id="rId1"/>
+    <sheet name="aboutUs" sheetId="2" r:id="rId2"/>
+    <sheet name="course" sheetId="3" r:id="rId3"/>
+    <sheet name="announcement" sheetId="4" r:id="rId4"/>
+    <sheet name="attachments" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="67">
+  <si>
+    <t>icon</t>
+  </si>
+  <si>
+    <t>websiteTitle</t>
+  </si>
+  <si>
+    <t>middleLogo</t>
+  </si>
+  <si>
+    <t>heroBg</t>
+  </si>
+  <si>
+    <t>hero1Title</t>
+  </si>
+  <si>
+    <t>hero1Text</t>
+  </si>
+  <si>
+    <t>hero2Title</t>
+  </si>
+  <si>
+    <t>hero2Text</t>
+  </si>
+  <si>
+    <t>hero3Title</t>
+  </si>
+  <si>
+    <t>hero3Text</t>
+  </si>
+  <si>
+    <t>contactTitle</t>
+  </si>
+  <si>
+    <t>contactIntro</t>
+  </si>
+  <si>
+    <t>contactPhone</t>
+  </si>
+  <si>
+    <t>contactEmail</t>
+  </si>
+  <si>
+    <t>contactAddress</t>
+  </si>
+  <si>
+    <t>footerAddress</t>
+  </si>
+  <si>
+    <t>footerPhone1</t>
+  </si>
+  <si>
+    <t>footerPhone2</t>
+  </si>
+  <si>
+    <t>footerEmail</t>
+  </si>
+  <si>
+    <t>dataImages\favicon.png</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>dataImages\middleLogo.png</t>
+  </si>
+  <si>
+    <t>dataImages\BG.png</t>
+  </si>
+  <si>
+    <t>打造你的亮眼未來</t>
+  </si>
+  <si>
+    <t>以實作為核心的課程設計，搭配產業導師與校友網絡，讓學習更有方向、就業更有把握。</t>
+  </si>
+  <si>
+    <t>從興趣到專長的完整路徑</t>
+  </si>
+  <si>
+    <t>小班互動、實戰專案、跨域學習，打造一條真正能產生作品與成果的學習旅程。</t>
+  </si>
+  <si>
+    <t>連結產學、看見成長</t>
+  </si>
+  <si>
+    <t>我們提供研究資源、實習機會與業界連結，協助你在學期間建立作品集與專業人脈。</t>
+  </si>
+  <si>
+    <t>聯絡我們</t>
+  </si>
+  <si>
+    <t>如有課程或合作需求，歡迎留下訊息，我們將盡快與你聯繫。</t>
+  </si>
+  <si>
+    <t>+880 20 5784 3248</t>
+  </si>
+  <si>
+    <t>yourmail@email.com</t>
+  </si>
+  <si>
+    <t>71 Shelton Street&lt;br&gt;London WC2H 9JQ England</t>
+  </si>
+  <si>
+    <t>23621 15 Mile Rd #C104, Clinton MI, 48035, New York, USA</t>
+  </si>
+  <si>
+    <t>+1 (2) 345 6789</t>
+  </si>
+  <si>
+    <t>contact@yourdomain.com</t>
+  </si>
+  <si>
+    <t>MainTitle</t>
+  </si>
+  <si>
+    <t>LongIntro</t>
+  </si>
+  <si>
+    <t>ShortIntro</t>
+  </si>
+  <si>
+    <t>BackgroundPic</t>
+  </si>
+  <si>
+    <t>AboutUsPic</t>
+  </si>
+  <si>
+    <t>Founder</t>
+  </si>
+  <si>
+    <t>FounderIntroduction</t>
+  </si>
+  <si>
+    <t>FounderPic</t>
+  </si>
   <si>
     <t>主標題</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>icon</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dataImages\aboutUs\success-story.jpg</t>
   </si>
   <si>
     <t>創辦人</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>創辦人圖片</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>創辦人介紹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MainTitle</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BackgroundPic</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BigPic1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Founder</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FounderPic</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FounderIntroduction</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>websiteTitle</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>dataImages\aboutUs\success-story.jpg</t>
-  </si>
-  <si>
-    <t>LongIntro</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ShortIntro</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Title</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>middleLogo</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>dataImages\middleLogo.png</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>shortIntro</t>
+  </si>
+  <si>
+    <t>Img</t>
+  </si>
+  <si>
+    <t>Ai course</t>
+  </si>
+  <si>
+    <t>st about ai</t>
+  </si>
+  <si>
+    <t>dataImages\ShockIcon.png</t>
+  </si>
+  <si>
+    <t>Train course</t>
+  </si>
+  <si>
+    <t>about train</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>shortText</t>
+  </si>
+  <si>
+    <t>DetailText</t>
+  </si>
+  <si>
+    <t>New!!!</t>
+  </si>
+  <si>
+    <t>short new test</t>
+  </si>
+  <si>
+    <t>this is the detail</t>
+  </si>
+  <si>
+    <t>New2!!!</t>
+  </si>
+  <si>
+    <t>short new2 test</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>dataAttachments\Calculus_Homework_5.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="新細明體"/>
       <family val="2"/>
-      <charset val="136"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="新細明體"/>
-      <family val="2"/>
-      <charset val="136"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="新細明體"/>
-      <family val="2"/>
+      <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
@@ -158,28 +264,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
-    <cellStyle name="超連結" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -507,135 +603,373 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D563F2B-87E7-4475-823C-C6BA693017D8}">
-  <dimension ref="A1:C2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" customWidth="1"/>
+    <col min="11" max="11" width="16.44140625" customWidth="1"/>
+    <col min="12" max="12" width="27.33203125" customWidth="1"/>
+    <col min="13" max="13" width="20.109375" customWidth="1"/>
+    <col min="14" max="14" width="17.88671875" customWidth="1"/>
+    <col min="15" max="15" width="19.77734375" customWidth="1"/>
+    <col min="16" max="16" width="19" customWidth="1"/>
+    <col min="17" max="17" width="15.33203125" customWidth="1"/>
+    <col min="18" max="18" width="16" customWidth="1"/>
+    <col min="19" max="19" width="23.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" t="s">
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
       <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S2" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{1025D2D0-FEB9-405F-A577-4B55E6E69442}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:S2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC7D1D14-586A-4D43-8496-21307256CCED}">
-  <dimension ref="A1:J6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="10.44140625" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" customWidth="1"/>
-    <col min="6" max="6" width="6.77734375" customWidth="1"/>
-    <col min="9" max="9" width="12.88671875" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="E1" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" t="s">
+        <v>46</v>
       </c>
       <c r="H2" t="s">
-        <v>2</v>
+        <v>47</v>
       </c>
       <c r="I2" t="s">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="J2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B6" s="1"/>
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{0D8CF109-EFB4-4522-9A9D-9D8AADB9C198}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="F2" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="J2" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:J2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01C7D10-878C-4F39-891A-34496F598264}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:D3" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DA483C1-44DA-46B0-8A21-8AC1CA93E02B}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46046</v>
+      </c>
+      <c r="C2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46046</v>
+      </c>
+      <c r="C3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3">
+        <v>2222222222</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:E3" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1001</v>
+      </c>
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:B2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>